<commit_message>
write reporting log files
</commit_message>
<xml_diff>
--- a/trapper_data_report.xlsx
+++ b/trapper_data_report.xlsx
@@ -33746,7 +33746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -36947,6 +36947,836 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>45931</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>51.65212017238942</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>-124.4085851818315</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>10010009.JPG</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2025-10-01%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 51.652120172389424 -124.4085851818315%0D%A0Photo Name: 10010009.JPG"&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="n">
+        <v>45932.81792822917</v>
+      </c>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr"/>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="n">
+        <v>45926</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>51.65084284569738</v>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>-124.4020894349512</v>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2025-09-26%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 51.65084284569738 -124.40208943495117%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="n">
+        <v>45957.552582581</v>
+      </c>
+      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr"/>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr"/>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>45943</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>51.65174648764192</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>-124.4022208631934</v>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2025-10-13%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 51.651746487641915 -124.40222086319343%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="n">
+        <v>45957.55381864582</v>
+      </c>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>45979</v>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>51.825759</v>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>-121.661309</v>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2025-11-18%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 51.825759 -121.661309%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="n">
+        <v>45980.81844434028</v>
+      </c>
+      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr"/>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1km</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="n">
+        <v>45977</v>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>51.90355917568825</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>-122.0103286521498</v>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>TRACK</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr"/>
+      <c r="P90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="n">
+        <v>45987</v>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>51.93760236780627</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>-122.0162546602725</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr"/>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>TRACK</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>51.95065913261133</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>-122.0204832126591</v>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr"/>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>TRACK</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr"/>
+      <c r="P92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>51.95950877575414</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>-122.0416357130915</v>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr"/>
+      <c r="P93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="n">
+        <v>46018</v>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>51.95464627822111</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>-122.0666975063477</v>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>TRACK</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr"/>
+      <c r="P94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>53.83751157650119</v>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>-124.2313698924538</v>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-01-16%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 53.837511576501186 -124.23136989245383%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="n">
+        <v>46039.46589590277</v>
+      </c>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="n">
+        <v>46022</v>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>51.96212215333761</v>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>-122.1982278418771</v>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr"/>
+      <c r="P96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="n">
+        <v>46001</v>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>49.41623045641039</v>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>-123.5960595752057</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2025-12-10%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 49.41623045641039 -123.59605957520574%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="n">
+        <v>46041.94828915509</v>
+      </c>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>&lt;10km</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="n">
+        <v>46103</v>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>53.361198</v>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>-120.269997</v>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>IMG_9467.jpeg</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-03-22%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 53.361198 -120.269997%0D%A0Photo Name: IMG_9467.jpeg"&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="n">
+        <v>46103.69157703704</v>
+      </c>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr"/>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="n">
+        <v>46098</v>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>50.67913866491195</v>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>-119.0545202136211</v>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-03-17%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 50.67913866491195 -119.05452021362107%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="n">
+        <v>46105.17767163194</v>
+      </c>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr"/>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="n">
+        <v>46116</v>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>53.60353247521391</v>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>-122.9489864017633</v>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-04-04%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 53.60353247521391 -122.94898640176334%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="n">
+        <v>46120.24911616898</v>
+      </c>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="n">
+        <v>46147</v>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>50.67944932433205</v>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>-119.0545349113452</v>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr"/>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-05-05%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 50.679449324332055 -119.05453491134521%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="n">
+        <v>46147.95886540508</v>
+      </c>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr"/>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="n">
+        <v>46154</v>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>53.49343265655232</v>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>-123.5488064211401</v>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-05-12%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 53.493432656552315 -123.54880642114013%0D%A0Photo Name: "&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="n">
+        <v>46157.66040622685</v>
+      </c>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr"/>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>49.89604995704579</v>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>-119.500441527063</v>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>20260524_215232.jpg</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr"/>
+      <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-05-24%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 49.89604995704579 -119.500441527063%0D%A0Photo Name: 20260524_215232.jpg"&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="n">
+        <v>46167.24132527777</v>
+      </c>
+      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr"/>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>&lt;100m</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>FISHER</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C104" s="2" t="n">
+        <v>50.73701252190629</v>
+      </c>
+      <c r="D104" s="2" t="n">
+        <v>-120.1529333680133</v>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>IMG_5683.png</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Not Reviewed</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>&lt;a href="mailto:?subject=Fisher Observation Response Summary&amp;body=Species: FISHER%0D%A0When did you see the fisher? 2026-06-26%0D%A0Observation Type: VISUAL%0D%A0Where did you see the fisher? (lat, long): 50.737012521906294 -120.15293336801328%0D%A0Photo Name: IMG_5683.png"&gt;Email me the response summary&lt;/a&gt;</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="n">
+        <v>46204.97825337963</v>
+      </c>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>VISUAL</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr"/>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1km</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>